<commit_message>
final changes done, reports issue done and light theme fixed
</commit_message>
<xml_diff>
--- a/analytics/reports/ticketflicks_analytics_report.xlsx
+++ b/analytics/reports/ticketflicks_analytics_report.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>₹7,500.00</t>
+          <t>₹8,781.00</t>
         </is>
       </c>
     </row>
@@ -483,7 +483,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>₹500.00</t>
+          <t>₹585.40</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -505,7 +505,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
@@ -635,7 +635,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>1.5</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>₹1,250.00</t>
+          <t>₹878.10</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-03-05 00:24:33</t>
+          <t>2026-03-06 00:42:26</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -717,18 +717,38 @@
           <t>total_spent</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>6978a7149c3b5dc208ba268d</t>
+          <t>69a9c33fc33095b555984eeb</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>2000</v>
+        <v>1317</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Kabir Verma</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>customer6990@example.com</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -743,6 +763,16 @@
       <c r="C3" t="n">
         <v>1100</v>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Aarav Sharma</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>aaravsharma683@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -756,6 +786,16 @@
       <c r="C4" t="n">
         <v>1100</v>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Priya Patel</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>priyapatel282@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -769,6 +809,16 @@
       <c r="C5" t="n">
         <v>1100</v>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Aditya Verma</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>adityaverma745@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -782,6 +832,16 @@
       <c r="C6" t="n">
         <v>1100</v>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Neha Reddy</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nehareddy847@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -794,6 +854,108 @@
       </c>
       <c r="C7" t="n">
         <v>1100</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Rohan Desai</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>rohandesai204@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>69a9c33fc33095b555984ee8</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>618</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Diya Patel</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>customer6187@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>69a9c33fc33095b555984ee9</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>510</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Rohan Gupta</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>customer5689@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>69a9c33fc33095b555984eea</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>447</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Neha Singh</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>customer8107@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>69a9c33fc33095b555984ee7</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>389</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Aarav Sharma</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>customer2246@example.com</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -807,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -829,24 +991,57 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46083</v>
+        <v>46082</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>800</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46084</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
         <v>46085</v>
       </c>
-      <c r="B3" t="n">
-        <v>14</v>
-      </c>
-      <c r="C3" t="n">
-        <v>6700</v>
+      <c r="B5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C5" t="n">
+        <v>6118</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46086</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>389</v>
       </c>
     </row>
   </sheetData>
@@ -913,95 +1108,103 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>69a54b5c442b1451606b555d</t>
+          <t>69a87f227287871ef58e1da7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6978a7149c3b5dc208ba268d</t>
+          <t>69a87f227287871ef58e1d98</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>69a3358c179d8faa9ad34e40</t>
+          <t>69a8780375d9b89273915b89</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>800</v>
+        <v>550</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>cancelled</t>
+          <t>confirmed</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>stripe</t>
+        </is>
+      </c>
       <c r="I2" s="1" t="n">
-        <v>46083.35663039351</v>
+        <v>46085.78558711806</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>69a7f0d6065c17c59119001b</t>
+          <t>69a87f227287871ef58e1dae</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>6978a7149c3b5dc208ba268d</t>
+          <t>69a87f227287871ef58e1d98</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>69a6cb1affde849a03dbfbc5</t>
+          <t>69a877ff75d9b89273915b2c</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>750</v>
+        <v>550</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>cancelled</t>
+          <t>confirmed</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>5</v>
-      </c>
-      <c r="H3" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>stripe</t>
+        </is>
+      </c>
       <c r="I3" s="1" t="n">
-        <v>46085.3639657176</v>
+        <v>46085.78558873843</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>69a80158ef903b13a6931eea</t>
+          <t>69a87f227287871ef58e1db5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6978a7149c3b5dc208ba268d</t>
+          <t>69a87f227287871ef58e1d9a</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>69a6cb1affde849a03dbfbc2</t>
+          <t>69a8780175d9b89273915b4c</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>150</v>
+        <v>550</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1014,31 +1217,35 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>stripe</t>
+        </is>
+      </c>
       <c r="I4" s="1" t="n">
-        <v>46085.41287819445</v>
+        <v>46085.78558971065</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>69a80158ef903b13a6931eee</t>
+          <t>69a87f237287871ef58e1dbc</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6978a7149c3b5dc208ba268d</t>
+          <t>69a87f227287871ef58e1d9a</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>69a6cb1affde849a03dbfbc2</t>
+          <t>69a8780275d9b89273915b6a</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>150</v>
+        <v>550</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1051,31 +1258,35 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>stripe</t>
+        </is>
+      </c>
       <c r="I5" s="1" t="n">
-        <v>46085.41287850695</v>
+        <v>46085.78559078704</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>69a80158ef903b13a6931ef2</t>
+          <t>69a87f237287871ef58e1dc3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>6978a7149c3b5dc208ba268d</t>
+          <t>69a87f227287871ef58e1d9e</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>69a6cb1affde849a03dbfbc2</t>
+          <t>69a8780475d9b89273915ba6</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>150</v>
+        <v>550</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1088,27 +1299,31 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>stripe</t>
+        </is>
+      </c>
       <c r="I6" s="1" t="n">
-        <v>46085.41287925926</v>
+        <v>46085.78559186342</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1da7</t>
+          <t>69a87f237287871ef58e1dca</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1d98</t>
+          <t>69a87f227287871ef58e1d9e</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>69a8780375d9b89273915b89</t>
+          <t>69a8780775d9b89273915c00</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -1133,23 +1348,23 @@
         </is>
       </c>
       <c r="I7" s="1" t="n">
-        <v>46085.78558711806</v>
+        <v>46085.78559314815</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1dae</t>
+          <t>69a87f237287871ef58e1dd1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1d98</t>
+          <t>69a87f227287871ef58e1da0</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>69a877ff75d9b89273915b2c</t>
+          <t>69a877ff75d9b89273915b2b</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1174,23 +1389,23 @@
         </is>
       </c>
       <c r="I8" s="1" t="n">
-        <v>46085.78558873843</v>
+        <v>46085.78559429398</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1db5</t>
+          <t>69a87f237287871ef58e1dd8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1d9a</t>
+          <t>69a87f227287871ef58e1da0</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>69a8780175d9b89273915b4c</t>
+          <t>69a8780575d9b89273915bc1</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1215,23 +1430,23 @@
         </is>
       </c>
       <c r="I9" s="1" t="n">
-        <v>46085.78558971065</v>
+        <v>46085.78559533565</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1dbc</t>
+          <t>69a87f237287871ef58e1ddf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1d9a</t>
+          <t>69a87f227287871ef58e1da2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>69a8780275d9b89273915b6a</t>
+          <t>69a8780475d9b89273915ba6</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1256,23 +1471,23 @@
         </is>
       </c>
       <c r="I10" s="1" t="n">
-        <v>46085.78559078704</v>
+        <v>46085.78559663195</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1dc3</t>
+          <t>69a87f237287871ef58e1de6</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1d9e</t>
+          <t>69a87f227287871ef58e1da2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>69a8780475d9b89273915ba6</t>
+          <t>69a8780875d9b89273915c1e</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1297,212 +1512,172 @@
         </is>
       </c>
       <c r="I11" s="1" t="n">
-        <v>46085.78559186342</v>
+        <v>46085.78559770833</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1dca</t>
+          <t>69a9c340c33095b555984eec</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1d9e</t>
+          <t>69a9c33fc33095b555984ee7</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>69a8780775d9b89273915c00</t>
+          <t>69a8780175d9b89273915b48</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>550</v>
+        <v>389</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>2</v>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>stripe</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" s="1" t="n">
-        <v>46085.78559314815</v>
+        <v>46086.74592653936</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1dd1</t>
+          <t>69a9c340c33095b555984eed</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1da0</t>
+          <t>69a9c33fc33095b555984ee8</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>69a877ff75d9b89273915b2b</t>
+          <t>69a8780675d9b89273915bec</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>550</v>
+        <v>618</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
         <v>2</v>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>stripe</t>
-        </is>
-      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" s="1" t="n">
-        <v>46085.78559429398</v>
+        <v>46085.74592653936</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1dd8</t>
+          <t>69a9c340c33095b555984eee</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1da0</t>
+          <t>69a9c33fc33095b555984ee9</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>69a8780575d9b89273915bc1</t>
+          <t>69a8780275d9b89273915b6d</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>550</v>
+        <v>510</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
         <v>2</v>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>stripe</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" s="1" t="n">
-        <v>46085.78559533565</v>
+        <v>46084.74592653936</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1ddf</t>
+          <t>69a9c340c33095b555984eef</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1da2</t>
+          <t>69a9c33fc33095b555984eea</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>69a8780475d9b89273915ba6</t>
+          <t>69a8780375d9b89273915b86</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>550</v>
+        <v>447</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
         <v>2</v>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>stripe</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" s="1" t="n">
-        <v>46085.78559663195</v>
+        <v>46083.74592653936</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1de6</t>
+          <t>69a9c340c33095b555984ef0</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1da2</t>
+          <t>69a9c33fc33095b555984eeb</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>69a8780875d9b89273915c1e</t>
+          <t>69a8780075d9b89273915b46</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>550</v>
+        <v>1317</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
         <v>2</v>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>stripe</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" s="1" t="n">
-        <v>46085.78559770833</v>
+        <v>46082.74592653936</v>
       </c>
     </row>
   </sheetData>
@@ -11537,7 +11712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12050,6 +12225,136 @@
       </c>
       <c r="F17" s="1" t="n">
         <v>46085.78558376157</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>69a9c33fc33095b555984ee7</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Aarav Sharma</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>customer2246@example.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="n">
+        <v>46086.74592559028</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>69a9c33fc33095b555984ee8</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Diya Patel</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>customer6187@example.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>46086.74592559028</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>69a9c33fc33095b555984ee9</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Rohan Gupta</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>customer5689@example.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="n">
+        <v>46086.74592559028</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>69a9c33fc33095b555984eea</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Neha Singh</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>customer8107@example.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>46086.74592559028</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>69a9c33fc33095b555984eeb</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kabir Verma</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>customer6990@example.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>46086.74592559028</v>
       </c>
     </row>
   </sheetData>
@@ -12131,78 +12436,106 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>69a54b5c442b1451606b555d</t>
+          <t>69a87f227287871ef58e1da7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Test Admin</t>
+          <t>Aarav Sharma</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>admin@test.com</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+          <t>aaravsharma683@gmail.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>In the Lost Lands</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PVR Forum Mall Koramangala</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>46086.70833333334</v>
+      </c>
       <c r="H2" t="n">
-        <v>800</v>
+        <v>550</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>cancelled</t>
+          <t>confirmed</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>46083</v>
+        <v>46085</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>69a7f0d6065c17c59119001b</t>
+          <t>69a87f227287871ef58e1dae</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Test Admin</t>
+          <t>Aarav Sharma</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>admin@test.com</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+          <t>aaravsharma683@gmail.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Thunderbolts*</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>INOX R-City Mall</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>46086.33333333334</v>
+      </c>
       <c r="H3" t="n">
-        <v>750</v>
+        <v>550</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>cancelled</t>
+          <t>confirmed</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>46085</v>
@@ -12211,25 +12544,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>69a80158ef903b13a6931eea</t>
+          <t>69a87f227287871ef58e1db5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Test Admin</t>
+          <t>Priya Patel</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>admin@test.com</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+          <t>priyapatel282@gmail.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Devara: Part 1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PVR Directors Cut Select City Walk</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>46086.58333333334</v>
+      </c>
       <c r="H4" t="n">
-        <v>150</v>
+        <v>550</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -12242,7 +12589,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>46085</v>
@@ -12251,25 +12598,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>69a80158ef903b13a6931eee</t>
+          <t>69a87f237287871ef58e1dbc</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Test Admin</t>
+          <t>Priya Patel</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>admin@test.com</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+          <t>priyapatel282@gmail.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Devara: Part 1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>INOX DLF Promenade</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>46086.58333333334</v>
+      </c>
       <c r="H5" t="n">
-        <v>150</v>
+        <v>550</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -12282,7 +12643,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>46085</v>
@@ -12291,25 +12652,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>69a80158ef903b13a6931ef2</t>
+          <t>69a87f237287871ef58e1dc3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Test Admin</t>
+          <t>Aditya Verma</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>admin@test.com</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+          <t>adityaverma745@gmail.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Devara: Part 1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PVR ICONX GVK One Mall</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>46086.58333333334</v>
+      </c>
       <c r="H6" t="n">
-        <v>150</v>
+        <v>550</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -12322,7 +12697,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L6" s="2" t="n">
         <v>46085</v>
@@ -12331,36 +12706,36 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1da7</t>
+          <t>69a87f237287871ef58e1dca</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Aarav Sharma</t>
+          <t>Aditya Verma</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>aaravsharma683@gmail.com</t>
+          <t>adityaverma745@gmail.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>In the Lost Lands</t>
+          <t>Devara: Part 1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PVR Forum Mall Koramangala</t>
+          <t>PVR Phoenix Marketcity Pune</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="G7" s="1" t="n">
-        <v>46086.70833333334</v>
+        <v>46086.58333333334</v>
       </c>
       <c r="H7" t="n">
         <v>550</v>
@@ -12385,22 +12760,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1dae</t>
+          <t>69a87f237287871ef58e1dd1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Aarav Sharma</t>
+          <t>Neha Reddy</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>aaravsharma683@gmail.com</t>
+          <t>nehareddy847@gmail.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Thunderbolts*</t>
+          <t>Mission: Impossible - The Final Reckoning</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -12414,7 +12789,7 @@
         </is>
       </c>
       <c r="G8" s="1" t="n">
-        <v>46086.33333333334</v>
+        <v>46086.1875</v>
       </c>
       <c r="H8" t="n">
         <v>550</v>
@@ -12439,36 +12814,36 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>69a87f227287871ef58e1db5</t>
+          <t>69a87f237287871ef58e1dd8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Priya Patel</t>
+          <t>Neha Reddy</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>priyapatel282@gmail.com</t>
+          <t>nehareddy847@gmail.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Devara: Part 1</t>
+          <t>Mission: Impossible - The Final Reckoning</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>PVR Directors Cut Select City Walk</t>
+          <t>PVR VR Chennai</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="G9" s="1" t="n">
-        <v>46086.58333333334</v>
+        <v>46086.1875</v>
       </c>
       <c r="H9" t="n">
         <v>550</v>
@@ -12493,17 +12868,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1dbc</t>
+          <t>69a87f237287871ef58e1ddf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Priya Patel</t>
+          <t>Rohan Desai</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>priyapatel282@gmail.com</t>
+          <t>rohandesai204@gmail.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -12513,12 +12888,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>INOX DLF Promenade</t>
+          <t>PVR ICONX GVK One Mall</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="G10" s="1" t="n">
@@ -12547,17 +12922,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1dc3</t>
+          <t>69a87f237287871ef58e1de6</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Aditya Verma</t>
+          <t>Rohan Desai</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>adityaverma745@gmail.com</t>
+          <t>rohandesai204@gmail.com</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -12567,12 +12942,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>PVR ICONX GVK One Mall</t>
+          <t>PVR Acropolis Mall</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Kolkata</t>
         </is>
       </c>
       <c r="G11" s="1" t="n">
@@ -12601,104 +12976,96 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1dca</t>
+          <t>69a9c340c33095b555984eec</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Aditya Verma</t>
+          <t>Aarav Sharma</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>adityaverma745@gmail.com</t>
+          <t>customer2246@example.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Devara: Part 1</t>
+          <t>Until Dawn</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PVR Phoenix Marketcity Pune</t>
+          <t>INOX R-City Mall</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46086.58333333334</v>
+        <v>46091.70833333334</v>
       </c>
       <c r="H12" t="n">
-        <v>550</v>
+        <v>389</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
         <v>2</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>46085</v>
+        <v>46086</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1dd1</t>
+          <t>69a9c340c33095b555984eed</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Neha Reddy</t>
+          <t>Diya Patel</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>nehareddy847@gmail.com</t>
+          <t>customer6187@example.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Mission: Impossible - The Final Reckoning</t>
+          <t>Until Dawn</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>INOX R-City Mall</t>
+          <t>Sathyam Cinemas</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46086.1875</v>
+        <v>46088.58333333334</v>
       </c>
       <c r="H13" t="n">
-        <v>550</v>
+        <v>618</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
         <v>2</v>
       </c>
@@ -12709,125 +13076,117 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1dd8</t>
+          <t>69a9c340c33095b555984eee</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Neha Reddy</t>
+          <t>Rohan Gupta</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>nehareddy847@gmail.com</t>
+          <t>customer5689@example.com</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Mission: Impossible - The Final Reckoning</t>
+          <t>Lilo &amp; Stitch</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>PVR VR Chennai</t>
+          <t>INOX DLF Promenade</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46086.1875</v>
+        <v>46087.33333333334</v>
       </c>
       <c r="H14" t="n">
-        <v>550</v>
+        <v>510</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="n">
         <v>2</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>46085</v>
+        <v>46084</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1ddf</t>
+          <t>69a9c340c33095b555984eef</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Rohan Desai</t>
+          <t>Neha Singh</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>rohandesai204@gmail.com</t>
+          <t>customer8107@example.com</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Devara: Part 1</t>
+          <t>Thunderbolts*</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>PVR ICONX GVK One Mall</t>
+          <t>PVR Forum Mall Koramangala</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46086.58333333334</v>
+        <v>46086.33333333334</v>
       </c>
       <c r="H15" t="n">
-        <v>550</v>
+        <v>447</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
         <v>2</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>46085</v>
+        <v>46083</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>69a87f237287871ef58e1de6</t>
+          <t>69a9c340c33095b555984ef0</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Rohan Desai</t>
+          <t>Kabir Verma</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>rohandesai204@gmail.com</t>
+          <t>customer6990@example.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -12837,35 +13196,31 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PVR Acropolis Mall</t>
+          <t>INOX R-City Mall</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46086.58333333334</v>
+        <v>46091.45833333334</v>
       </c>
       <c r="H16" t="n">
-        <v>550</v>
+        <v>1317</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
         <v>2</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>46085</v>
+        <v>46082</v>
       </c>
     </row>
   </sheetData>
@@ -12879,7 +13234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12911,13 +13266,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>3300</v>
+        <v>4617</v>
       </c>
       <c r="D2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -12939,17 +13294,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>In the Lost Lands</t>
+          <t>Until Dawn</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>550</v>
+        <v>1007</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -12959,12 +13314,44 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>997</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>In the Lost Lands</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C6" t="n">
         <v>550</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Lilo &amp; Stitch</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>510</v>
+      </c>
+      <c r="D7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -12979,7 +13366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12990,15 +13377,20 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>bookings</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>revenue</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>seats_sold</t>
         </is>
@@ -13010,14 +13402,19 @@
           <t>INOX R-City Mall</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>2</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>1100</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>2806</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -13026,13 +13423,18 @@
           <t>PVR ICONX GVK One Mall</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>1100</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>4</v>
       </c>
     </row>
@@ -13042,93 +13444,144 @@
           <t>INOX DLF Promenade</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>1</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>550</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1060</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PVR Acropolis Mall</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
+          <t>PVR Forum Mall Koramangala</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>550</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>997</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PVR Directors Cut Select City Walk</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+          <t>Sathyam Cinemas</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" t="n">
-        <v>550</v>
-      </c>
       <c r="D6" t="n">
+        <v>618</v>
+      </c>
+      <c r="E6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PVR Forum Mall Koramangala</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+          <t>PVR Acropolis Mall</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>550</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PVR Phoenix Marketcity Pune</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+          <t>PVR Directors Cut Select City Walk</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>1</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>550</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>PVR Phoenix Marketcity Pune</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>550</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>PVR VR Chennai</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>1</v>
       </c>
-      <c r="C9" t="n">
+      <c r="D10" t="n">
         <v>550</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E10" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>